<commit_message>
Actualización automática: proyectos, cambios y dashboard
</commit_message>
<xml_diff>
--- a/data/watchlist_enriched.xlsx
+++ b/data/watchlist_enriched.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=15262&amp;prmBOLETIN=14767-03</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=14767</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=13644&amp;prmBOLETIN=13098-24</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=13098</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17258&amp;prmBOLETIN=16686-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16686</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=18138&amp;prmBOLETIN=17499-24</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17499</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=18783&amp;prmBOLETIN=18119-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=18119</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16257&amp;prmBOLETIN=15725-13</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15725</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16227&amp;prmBOLETIN=15694-34</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15694</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16416&amp;prmBOLETIN=15869-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15869</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17940&amp;prmBOLETIN=17307-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17307</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16473&amp;prmBOLETIN=15935-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15935</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16659&amp;prmBOLETIN=16112-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16112</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16563&amp;prmBOLETIN=16021-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16021</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17429&amp;prmBOLETIN=16821-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16821</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16950&amp;prmBOLETIN=16387-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16387</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17732&amp;prmBOLETIN=17112-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17112</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17940&amp;prmBOLETIN=17307-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17307</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/proyectosdeley/tramitacion.aspx?prmID=18265&amp;prmBOLETIN=17618-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17618</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=18447&amp;prmBOLETIN=17795-19</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17795</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=18682&amp;prmBOLETIN=18019-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=18019</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17292&amp;prmBOLETIN=16718-04</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16718</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16885&amp;prmBOLETIN=16329-04</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16329</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17086&amp;prmBOLETIN=16520-04</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16520</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17142&amp;prmBOLETIN=16575-04</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16575</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=17870&amp;prmBOLETIN=17241-17</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=17241</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=15766&amp;prmBOLETIN=15256-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15256</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16698&amp;prmBOLETIN=16146-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16146</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16611&amp;prmBOLETIN=16068-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16068</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=16570&amp;prmBOLETIN=16030-16</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16030</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=15565&amp;prmBOLETIN=15056-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15056</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=12838&amp;prmBOLETIN=12314-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=12314</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=13924&amp;prmBOLETIN=13383-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=13383</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=14260&amp;prmBOLETIN=13698-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=13698</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=15746&amp;prmBOLETIN=15234-06</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=15234</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.camara.cl/legislacion/ProyectosDeLey/tramitacion.aspx?prmID=14260&amp;prmBOLETIN=13698-07</t>
+          <t>https://tramitacion.senado.cl/wspublico/tramitacion.php?boletin=16393</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">

</xml_diff>